<commit_message>
Ajusta el plan rodilla a la segunda ronda de la revision
- Bici: vuelve la nota original (lo primero que se quita en un brote). Entra
  el viernes de S4 solo si S2 y S3 no tuvieron sesiones en Retroceder; se
  quita por un brote o un fallo atribuido a ella y vuelve tras una semana
  entera en verde. Hoy la muestra como "Sin bici (quitada)".
- Novedad: solo si esa manana esta igual o mejor que la referencia (la del
  mismo dia de la semana anterior), no que el dia anterior.
- Atribucion: una manana peor va a la ultima novedad aun no validada (sin
  sus dos mananas en verde); sin ninguna, brote. Sin ventana de 7 dias.
- Carrera despues del viaje: N7 18', N8 25' y N9 30' seguidos.
- Excel sin formulas matriciales (Excel para iPhone las calculaba a 0): la
  tabla de series por grupo y la peor manana semanal pasan a formulas
  normales. verify_plan lo comprueba y la evaluacion da 52 -> 88.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Plan_8sem_vol_definitivo_con_cardio.xlsx
+++ b/Plan_8sem_vol_definitivo_con_cardio.xlsx
@@ -9215,35 +9215,35 @@
         <v/>
       </c>
       <c r="C73" s="77">
-        <f t="array" ref="C73:C73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C25,FIND(" ",C25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C26,FIND(" ",C26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C28,FIND(" ",C28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C51,FIND(" ",C51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C52,FIND(" ",C52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C53,FIND(" ",C53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D73" s="77">
-        <f t="array" ref="D73:D73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D25,FIND(" ",D25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D26,FIND(" ",D26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D28,FIND(" ",D28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D51,FIND(" ",D51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D52,FIND(" ",D52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D53,FIND(" ",D53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E73" s="77">
-        <f t="array" ref="E73:E73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E25,FIND(" ",E25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E26,FIND(" ",E26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E28,FIND(" ",E28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E51,FIND(" ",E51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E52,FIND(" ",E52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E53,FIND(" ",E53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F73" s="77">
-        <f t="array" ref="F73:F73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F25,FIND(" ",F25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F26,FIND(" ",F26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F28,FIND(" ",F28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F51,FIND(" ",F51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F52,FIND(" ",F52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F53,FIND(" ",F53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G73" s="77">
-        <f t="array" ref="G73:G73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G25,FIND(" ",G25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G26,FIND(" ",G26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G28,FIND(" ",G28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G51,FIND(" ",G51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G52,FIND(" ",G52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G53,FIND(" ",G53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H73" s="77">
-        <f t="array" ref="H73:H73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H25,FIND(" ",H25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H26,FIND(" ",H26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H28,FIND(" ",H28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H51,FIND(" ",H51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H52,FIND(" ",H52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H53,FIND(" ",H53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I73" s="77">
-        <f t="array" ref="I73:I73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I25,FIND(" ",I25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I26,FIND(" ",I26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I28,FIND(" ",I28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I51,FIND(" ",I51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I52,FIND(" ",I52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I53,FIND(" ",I53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J73" s="77">
-        <f t="array" ref="J73:J73">SUM(($B$3:$B$63="Espalda")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J25,FIND(" ",J25&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J26,FIND(" ",J26&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J28,FIND(" ",J28&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J51,FIND(" ",J51&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J52,FIND(" ",J52&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J53,FIND(" ",J53&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K73" s="77" t="n"/>
@@ -9259,35 +9259,35 @@
         <v/>
       </c>
       <c r="C74" s="77">
-        <f t="array" ref="C74:C74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C16,FIND(" ",C16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C18,FIND(" ",C18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C50,FIND(" ",C50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D74" s="77">
-        <f t="array" ref="D74:D74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D16,FIND(" ",D16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D18,FIND(" ",D18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D50,FIND(" ",D50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E74" s="77">
-        <f t="array" ref="E74:E74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E16,FIND(" ",E16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E18,FIND(" ",E18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E50,FIND(" ",E50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F74" s="77">
-        <f t="array" ref="F74:F74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F16,FIND(" ",F16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F18,FIND(" ",F18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F50,FIND(" ",F50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G74" s="77">
-        <f t="array" ref="G74:G74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G16,FIND(" ",G16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G18,FIND(" ",G18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G50,FIND(" ",G50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H74" s="77">
-        <f t="array" ref="H74:H74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H16,FIND(" ",H16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H18,FIND(" ",H18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H50,FIND(" ",H50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I74" s="77">
-        <f t="array" ref="I74:I74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I16,FIND(" ",I16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I18,FIND(" ",I18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I50,FIND(" ",I50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J74" s="77">
-        <f t="array" ref="J74:J74">SUM(($B$3:$B$63="Pecho")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J16,FIND(" ",J16&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J18,FIND(" ",J18&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J50,FIND(" ",J50&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K74" s="77" t="n"/>
@@ -9303,35 +9303,35 @@
         <v/>
       </c>
       <c r="C75" s="77">
-        <f t="array" ref="C75:C75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C6,FIND(" ",C6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C8,FIND(" ",C8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C27,FIND(" ",C27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C47,FIND(" ",C47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D75" s="77">
-        <f t="array" ref="D75:D75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D6,FIND(" ",D6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D8,FIND(" ",D8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D27,FIND(" ",D27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D47,FIND(" ",D47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E75" s="77">
-        <f t="array" ref="E75:E75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E6,FIND(" ",E6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E8,FIND(" ",E8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E27,FIND(" ",E27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E47,FIND(" ",E47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F75" s="77">
-        <f t="array" ref="F75:F75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F6,FIND(" ",F6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F8,FIND(" ",F8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F27,FIND(" ",F27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F47,FIND(" ",F47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G75" s="77">
-        <f t="array" ref="G75:G75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G6,FIND(" ",G6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G8,FIND(" ",G8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G27,FIND(" ",G27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G47,FIND(" ",G47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H75" s="77">
-        <f t="array" ref="H75:H75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H6,FIND(" ",H6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H8,FIND(" ",H8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H27,FIND(" ",H27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H47,FIND(" ",H47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I75" s="77">
-        <f t="array" ref="I75:I75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I6,FIND(" ",I6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I8,FIND(" ",I8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I27,FIND(" ",I27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I47,FIND(" ",I47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J75" s="77">
-        <f t="array" ref="J75:J75">SUM(($B$3:$B$63="Hombro lat.")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J6,FIND(" ",J6&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J8,FIND(" ",J8&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J27,FIND(" ",J27&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J47,FIND(" ",J47&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K75" s="77" t="n"/>
@@ -9347,35 +9347,35 @@
         <v/>
       </c>
       <c r="C76" s="77">
-        <f t="array" ref="C76:C76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C30,FIND(" ",C30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D76" s="77">
-        <f t="array" ref="D76:D76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D30,FIND(" ",D30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E76" s="77">
-        <f t="array" ref="E76:E76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E30,FIND(" ",E30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F76" s="77">
-        <f t="array" ref="F76:F76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F30,FIND(" ",F30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G76" s="77">
-        <f t="array" ref="G76:G76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G30,FIND(" ",G30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H76" s="77">
-        <f t="array" ref="H76:H76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H30,FIND(" ",H30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I76" s="77">
-        <f t="array" ref="I76:I76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I30,FIND(" ",I30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J76" s="77">
-        <f t="array" ref="J76:J76">SUM(($B$3:$B$63="Hombro post.")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J30,FIND(" ",J30&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K76" s="77" t="n"/>
@@ -9391,35 +9391,35 @@
         <v/>
       </c>
       <c r="C77" s="77">
-        <f t="array" ref="C77:C77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C29,FIND(" ",C29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C31,FIND(" ",C31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C49,FIND(" ",C49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D77" s="77">
-        <f t="array" ref="D77:D77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D29,FIND(" ",D29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D31,FIND(" ",D31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D49,FIND(" ",D49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E77" s="77">
-        <f t="array" ref="E77:E77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E29,FIND(" ",E29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E31,FIND(" ",E31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E49,FIND(" ",E49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F77" s="77">
-        <f t="array" ref="F77:F77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F29,FIND(" ",F29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F31,FIND(" ",F31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F49,FIND(" ",F49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G77" s="77">
-        <f t="array" ref="G77:G77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G29,FIND(" ",G29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G31,FIND(" ",G31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G49,FIND(" ",G49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H77" s="77">
-        <f t="array" ref="H77:H77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H29,FIND(" ",H29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H31,FIND(" ",H31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H49,FIND(" ",H49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I77" s="77">
-        <f t="array" ref="I77:I77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I29,FIND(" ",I29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I31,FIND(" ",I31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I49,FIND(" ",I49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J77" s="77">
-        <f t="array" ref="J77:J77">SUM(($B$3:$B$63="Bíceps")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J29,FIND(" ",J29&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J31,FIND(" ",J31&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J49,FIND(" ",J49&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K77" s="77" t="n"/>
@@ -9435,35 +9435,35 @@
         <v/>
       </c>
       <c r="C78" s="77">
-        <f t="array" ref="C78:C78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C17,FIND(" ",C17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C19,FIND(" ",C19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C46,FIND(" ",C46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C48,FIND(" ",C48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D78" s="77">
-        <f t="array" ref="D78:D78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D17,FIND(" ",D17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D19,FIND(" ",D19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D46,FIND(" ",D46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D48,FIND(" ",D48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E78" s="77">
-        <f t="array" ref="E78:E78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E17,FIND(" ",E17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E19,FIND(" ",E19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E46,FIND(" ",E46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E48,FIND(" ",E48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F78" s="77">
-        <f t="array" ref="F78:F78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F17,FIND(" ",F17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F19,FIND(" ",F19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F46,FIND(" ",F46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F48,FIND(" ",F48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G78" s="77">
-        <f t="array" ref="G78:G78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G17,FIND(" ",G17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G19,FIND(" ",G19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G46,FIND(" ",G46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G48,FIND(" ",G48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H78" s="77">
-        <f t="array" ref="H78:H78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H17,FIND(" ",H17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H19,FIND(" ",H19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H46,FIND(" ",H46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H48,FIND(" ",H48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I78" s="77">
-        <f t="array" ref="I78:I78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I17,FIND(" ",I17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I19,FIND(" ",I19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I46,FIND(" ",I46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I48,FIND(" ",I48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J78" s="77">
-        <f t="array" ref="J78:J78">SUM(($B$3:$B$63="Tríceps")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J17,FIND(" ",J17&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J19,FIND(" ",J19&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J46,FIND(" ",J46&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J48,FIND(" ",J48&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K78" s="77" t="n"/>
@@ -9479,35 +9479,35 @@
         <v/>
       </c>
       <c r="C79" s="77">
-        <f t="array" ref="C79:C79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C12,FIND(" ",C12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C40,FIND(" ",C40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D79" s="77">
-        <f t="array" ref="D79:D79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D12,FIND(" ",D12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D40,FIND(" ",D40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E79" s="77">
-        <f t="array" ref="E79:E79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E12,FIND(" ",E12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E40,FIND(" ",E40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F79" s="77">
-        <f t="array" ref="F79:F79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F12,FIND(" ",F12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F40,FIND(" ",F40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G79" s="77">
-        <f t="array" ref="G79:G79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G12,FIND(" ",G12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G40,FIND(" ",G40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H79" s="77">
-        <f t="array" ref="H79:H79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H12,FIND(" ",H12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H40,FIND(" ",H40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I79" s="77">
-        <f t="array" ref="I79:I79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I12,FIND(" ",I12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I40,FIND(" ",I40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J79" s="77">
-        <f t="array" ref="J79:J79">SUM(($B$3:$B$63="Isquios")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J12,FIND(" ",J12&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J40,FIND(" ",J40&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K79" s="77" t="n"/>
@@ -9523,35 +9523,35 @@
         <v/>
       </c>
       <c r="C80" s="77">
-        <f t="array" ref="C80:C80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C20,FIND(" ",C20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C60,FIND(" ",C60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D80" s="77">
-        <f t="array" ref="D80:D80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D20,FIND(" ",D20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D60,FIND(" ",D60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E80" s="77">
-        <f t="array" ref="E80:E80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E20,FIND(" ",E20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E60,FIND(" ",E60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F80" s="77">
-        <f t="array" ref="F80:F80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F20,FIND(" ",F20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F60,FIND(" ",F60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G80" s="77">
-        <f t="array" ref="G80:G80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G20,FIND(" ",G20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G60,FIND(" ",G60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H80" s="77">
-        <f t="array" ref="H80:H80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H20,FIND(" ",H20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H60,FIND(" ",H60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I80" s="77">
-        <f t="array" ref="I80:I80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I20,FIND(" ",I20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I60,FIND(" ",I60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J80" s="77">
-        <f t="array" ref="J80:J80">SUM(($B$3:$B$63="Abs")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J20,FIND(" ",J20&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J60,FIND(" ",J60&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K80" s="77" t="n"/>
@@ -9567,35 +9567,35 @@
         <v/>
       </c>
       <c r="C81" s="77">
-        <f t="array" ref="C81:C81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C11,FIND(" ",C11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(C42,FIND(" ",C42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D81" s="77">
-        <f t="array" ref="D81:D81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D11,FIND(" ",D11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(D42,FIND(" ",D42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E81" s="77">
-        <f t="array" ref="E81:E81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E11,FIND(" ",E11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(E42,FIND(" ",E42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F81" s="77">
-        <f t="array" ref="F81:F81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F11,FIND(" ",F11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(F42,FIND(" ",F42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G81" s="77">
-        <f t="array" ref="G81:G81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G11,FIND(" ",G11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(G42,FIND(" ",G42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H81" s="77">
-        <f t="array" ref="H81:H81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H11,FIND(" ",H11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(H42,FIND(" ",H42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I81" s="77">
-        <f t="array" ref="I81:I81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I11,FIND(" ",I11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(I42,FIND(" ",I42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J81" s="77">
-        <f t="array" ref="J81:J81">SUM(($B$3:$B$63="Gemelos")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J11,FIND(" ",J11&amp;" ")-1)),0)+IFERROR(VALUE(LEFT(J42,FIND(" ",J42&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K81" s="77" t="n"/>
@@ -9611,35 +9611,35 @@
         <v/>
       </c>
       <c r="C82" s="77">
-        <f t="array" ref="C82:C82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(C$3:C$63,FIND(" ",C$3:C$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(C41,FIND(" ",C41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="D82" s="77">
-        <f t="array" ref="D82:D82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(D$3:D$63,FIND(" ",D$3:D$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(D41,FIND(" ",D41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="E82" s="77">
-        <f t="array" ref="E82:E82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(E$3:E$63,FIND(" ",E$3:E$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(E41,FIND(" ",E41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="F82" s="77">
-        <f t="array" ref="F82:F82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(F$3:F$63,FIND(" ",F$3:F$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(F41,FIND(" ",F41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="G82" s="77">
-        <f t="array" ref="G82:G82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(G$3:G$63,FIND(" ",G$3:G$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(G41,FIND(" ",G41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="H82" s="77">
-        <f t="array" ref="H82:H82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(H$3:H$63,FIND(" ",H$3:H$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(H41,FIND(" ",H41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="I82" s="77">
-        <f t="array" ref="I82:I82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(I$3:I$63,FIND(" ",I$3:I$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(I41,FIND(" ",I41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="J82" s="77">
-        <f t="array" ref="J82:J82">SUM(($B$3:$B$63="Aductores")*IFERROR(VALUE(LEFT(J$3:J$63,FIND(" ",J$3:J$63&amp;" ")-1)),0))</f>
+        <f>IFERROR(VALUE(LEFT(J41,FIND(" ",J41&amp;" ")-1)),0)</f>
         <v/>
       </c>
       <c r="K82" s="77" t="n"/>
@@ -10084,7 +10084,7 @@
       </c>
       <c r="K95" s="62" t="inlineStr">
         <is>
-          <t>No se hizo en S1: estímulo NUEVO [LÓGICA]. Entra en S4 (el viernes) solo si S2 y S3 cumplieron la regla; desde S5, martes y viernes. Sin Z3 en este bloque. En la regla de 48-72 h se mantiene si ya estaba introducida. Sillín alto (rodilla a 20-25° abajo), 85-90 rpm, sentado. 10 min fijos en el bloque; subir a 15 después del viaje, como novedad única.</t>
+          <t>No se hizo en S1: estímulo NUEVO [LÓGICA]. Entra en S4 (el viernes) solo si S2 y S3 cumplieron la regla; desde S5, martes y viernes. Sin Z3 en este bloque. Lo primero que se quita si hay brote. Sillín alto (rodilla a 20-25° abajo), 85-90 rpm, sentado. 10 min fijos en el bloque; subir a 15 después del viaje, como novedad única.</t>
         </is>
       </c>
     </row>
@@ -10199,7 +10199,7 @@
       </c>
       <c r="K97" s="62" t="inlineStr">
         <is>
-          <t>Formato: minutos trotando / minutos andando. Niveles: N1 8×(1'/2') · N2 6×(2'/1') · N3 4×(4'/1') · N4 4×(5'/1') · N5 3×(8'/1') · N6 2×(12'/1') · N7 30' seguidos (después del viaje). N5 es un nivel intermedio para que el tramo continuo más largo no crezca más de un 50 % por nivel (5 → 8 → 12 min) [LÓGICA]. El calendario marca el máximo de cada semana; el nivel real sale del semáforo: Avanzar = +1, Mantener = el mismo, Retroceder = −1. Nivel nuevo solo si esa mañana estás igual o mejor. 5 min andando antes; llano y firme. Regla de carrera: Retroceder si pasas de 2/10 durante, no vuelves al nivel previo en ≤60 min o la mañana siguiente estás peor; Mantener si cumple pero el peor valor 24-48 h supera la referencia; Avanzar si cumple y el peor 24-48 h ≤ referencia [EVIDENCIA de uso: TREK Education, basada en Esculier; no comparada con otros umbrales]. Cadencia +5-10% opcional [EVIDENCIA mixta: Bramah 2019, serie de 12 corredores con mejora de dolor y función mantenida a 3 meses; Esculier 2018, sin beneficio extra sobre la educación].</t>
+          <t>Formato: minutos trotando / minutos andando. Niveles: N1 8×(1'/2') · N2 6×(2'/1') · N3 4×(4'/1') · N4 4×(5'/1') · N5 3×(8'/1') · N6 2×(12'/1'); después del viaje, N7 18' · N8 25' · N9 30' seguidos. Desde N4 el tramo continuo más largo crece como mucho un 50 % por nivel (5 → 8 → 12 → 18 → 25 → 30 min); de N1 a N3 se dobla porque los tramos son muy cortos [LÓGICA]. El calendario marca el máximo de cada semana; el nivel real sale del semáforo: Avanzar = +1, Mantener = el mismo, Retroceder = −1. Nivel nuevo solo si esa mañana estás igual o mejor. 5 min andando antes; llano y firme. Regla de carrera: Retroceder si pasas de 2/10 durante, no vuelves al nivel previo en ≤60 min o la mañana siguiente estás peor; Mantener si cumple pero el peor valor 24-48 h supera la referencia; Avanzar si cumple y el peor 24-48 h ≤ referencia [EVIDENCIA de uso: TREK Education, basada en Esculier; no comparada con otros umbrales]. Cadencia +5-10% opcional [EVIDENCIA mixta: Bramah 2019, serie de 12 corredores con mejora de dolor y función mantenida a 3 meses; Esculier 2018, sin beneficio extra sobre la educación].</t>
         </is>
       </c>
     </row>
@@ -10421,7 +10421,7 @@
     <row r="106" ht="30.75" customHeight="1" s="52">
       <c r="A106" s="67" t="inlineStr">
         <is>
-          <t>Novedades [LÓGICA]: una por día y validada a las 24 y 48 h antes de repetirla. Lunes: escalón o reps (prensa) · miércoles: nivel de carrera · viernes de S4: bici. Solo si esa mañana estás igual o mejor. El calendario marca el máximo de cada semana; el nivel real sale del semáforo: Avanzar = nivel +1 (sin pasar del calendario), Mantener = el mismo, Retroceder = nivel −1. Lo validado se repite: el jueves usa la profundidad del lunes y el domingo repite el nivel del miércoles.</t>
+          <t>Novedades [LÓGICA]: una por día y validada a las 24 y 48 h antes de repetirla. Lunes: escalón o reps (prensa) · miércoles: nivel de carrera · viernes de S4: bici. Solo si esa mañana estás igual o mejor que la referencia (la mañana del mismo día de la semana anterior; en S3, la primera medición de S2), no que el día anterior: así un empeoramiento lento también salta. El calendario marca el máximo de cada semana; el nivel real sale del semáforo: Avanzar = nivel +1 (sin pasar del calendario), Mantener = el mismo, Retroceder = nivel −1. Lo validado se repite: el jueves usa la profundidad del lunes y el domingo repite el nivel del miércoles.</t>
         </is>
       </c>
       <c r="B106" s="56" t="n"/>
@@ -10489,7 +10489,7 @@
     <row r="110" ht="18" customHeight="1" s="52">
       <c r="A110" s="67" t="inlineStr">
         <is>
-          <t>Retroceso y brote [LÓGICA]: si una medición falla, se retrocede solo la última novedad anterior a ella (p. ej., jueves bien y viernes peor → se retrocede la carrera del miércoles y el escalón se mantiene); si tras el retroceso la siguiente medición vuelve a fallar, se retrocede la novedad anterior, y así hacia atrás. Si falla sin ninguna novedad reciente, o fallan dos sesiones seguidas: 48-72 h solo isométricos (sentadilla española 5×45 s diaria), y la bici si ya estaba introducida; luego se retoma un escalón por debajo en todo.</t>
+          <t>Retroceso y brote [LÓGICA]: un dolor durante la sesión retrocede la escalera de esa sesión. Si una mañana sale peor, se retrocede la última novedad aún no validada (la que todavía no tiene en verde sus dos mañanas, 24 y 48 h; p. ej., jueves bien y viernes peor → se retrocede la carrera del miércoles y el escalón se mantiene); una novedad ya validada no se culpa. Si tras el retroceso vuelve a fallar, se retrocede la novedad anterior sin validar. Brote = un fallo sin ninguna novedad sin validar, o dos sesiones seguidas en Retroceder: lo primero que se quita es la bici; 48-72 h solo isométricos (sentadilla española 5×45 s diaria) y caminar, sin bici; luego se retoma un escalón por debajo en todo. La bici vuelve al nivel del calendario cuando lleves una semana entera en verde.</t>
         </is>
       </c>
       <c r="B110" s="56" t="n"/>
@@ -15290,7 +15290,7 @@
       <c r="C72" s="56" t="n"/>
       <c r="D72" s="57" t="n"/>
       <c r="E72" s="92">
-        <f t="array" ref="E72:E72">IF(COUNTIFS($C$5:$C$67,$A72,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A72)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I5:I11)=0,"",MAX(I5:I11))</f>
         <v/>
       </c>
       <c r="F72" s="92">
@@ -15325,7 +15325,7 @@
       <c r="C73" s="56" t="n"/>
       <c r="D73" s="57" t="n"/>
       <c r="E73" s="92">
-        <f t="array" ref="E73:E73">IF(COUNTIFS($C$5:$C$67,$A73,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A73)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I12:I18)=0,"",MAX(I12:I18))</f>
         <v/>
       </c>
       <c r="F73" s="92">
@@ -15360,7 +15360,7 @@
       <c r="C74" s="56" t="n"/>
       <c r="D74" s="57" t="n"/>
       <c r="E74" s="92">
-        <f t="array" ref="E74:E74">IF(COUNTIFS($C$5:$C$67,$A74,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A74)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I19:I25)=0,"",MAX(I19:I25))</f>
         <v/>
       </c>
       <c r="F74" s="92">
@@ -15395,7 +15395,7 @@
       <c r="C75" s="56" t="n"/>
       <c r="D75" s="57" t="n"/>
       <c r="E75" s="92">
-        <f t="array" ref="E75:E75">IF(COUNTIFS($C$5:$C$67,$A75,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A75)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I26:I32)=0,"",MAX(I26:I32))</f>
         <v/>
       </c>
       <c r="F75" s="92">
@@ -15430,7 +15430,7 @@
       <c r="C76" s="56" t="n"/>
       <c r="D76" s="57" t="n"/>
       <c r="E76" s="92">
-        <f t="array" ref="E76:E76">IF(COUNTIFS($C$5:$C$67,$A76,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A76)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I33:I39)=0,"",MAX(I33:I39))</f>
         <v/>
       </c>
       <c r="F76" s="92">
@@ -15465,7 +15465,7 @@
       <c r="C77" s="56" t="n"/>
       <c r="D77" s="57" t="n"/>
       <c r="E77" s="92">
-        <f t="array" ref="E77:E77">IF(COUNTIFS($C$5:$C$67,$A77,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A77)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I40:I46)=0,"",MAX(I40:I46))</f>
         <v/>
       </c>
       <c r="F77" s="92">
@@ -15500,7 +15500,7 @@
       <c r="C78" s="56" t="n"/>
       <c r="D78" s="57" t="n"/>
       <c r="E78" s="92">
-        <f t="array" ref="E78:E78">IF(COUNTIFS($C$5:$C$67,$A78,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A78)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I47:I53)=0,"",MAX(I47:I53))</f>
         <v/>
       </c>
       <c r="F78" s="92">
@@ -15535,7 +15535,7 @@
       <c r="C79" s="56" t="n"/>
       <c r="D79" s="57" t="n"/>
       <c r="E79" s="92">
-        <f t="array" ref="E79:E79">IF(COUNTIFS($C$5:$C$67,$A79,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A79)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I54:I60)=0,"",MAX(I54:I60))</f>
         <v/>
       </c>
       <c r="F79" s="92">
@@ -15570,7 +15570,7 @@
       <c r="C80" s="56" t="n"/>
       <c r="D80" s="57" t="n"/>
       <c r="E80" s="92">
-        <f t="array" ref="E80:E80">IF(COUNTIFS($C$5:$C$67,$A80,$I$5:$I$67,"&gt;=0")=0,"",MAX(IF(($C$5:$C$67=$A80)*ISNUMBER($I$5:$I$67),$I$5:$I$67)))</f>
+        <f>IF(COUNT(I61:I67)=0,"",MAX(I61:I67))</f>
         <v/>
       </c>
       <c r="F80" s="92">

</xml_diff>

<commit_message>
Pierna 2 de S2 el viernes 30/10 (el jueves 29/10, libre)
La cabecera de la pierna 2 solo cambia de día en S1 (S1=J): en S2 la app la
pone el viernes, el día en que se hizo, como ya decía «Seguimiento rodilla».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Plan_8sem_vol_definitivo_con_cardio.xlsx
+++ b/Plan_8sem_vol_definitivo_con_cardio.xlsx
@@ -7904,7 +7904,7 @@
     <row r="39" ht="19.5" customHeight="1" s="52">
       <c r="A39" s="65" t="inlineStr">
         <is>
-          <t>(V) Viernes  ·  Rehab + Isquios + Aductores  ·  test de fuerza S3 / S5 / S7 (+ opcional S8)  (desde S3; S1-S2 se hizo el jueves)</t>
+          <t>(V) Viernes  ·  Rehab + Isquios + Aductores  ·  test de fuerza S3 / S5 / S7 (+ opcional S8)  (desde S2; S1 se hizo el jueves; en S2, el viernes 30/10)</t>
         </is>
       </c>
       <c r="B39" s="56" t="n"/>
@@ -7919,7 +7919,7 @@
       <c r="K39" s="57" t="n"/>
       <c r="L39" s="106" t="inlineStr">
         <is>
-          <t>sesion;S1=J;S2=J</t>
+          <t>sesion;S1=J</t>
         </is>
       </c>
     </row>

</xml_diff>